<commit_message>
sync: update affiliate_products.xlsx (2 new promo links)
</commit_message>
<xml_diff>
--- a/affiliate_products.xlsx
+++ b/affiliate_products.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="97">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="105">
   <si>
     <t>No</t>
   </si>
@@ -323,12 +323,44 @@
 📅 22 พ.ค. 69 - 8 มิ.ย. 69
 ลงทะเบียน และช้อปอัลบั้มไปหาน้องกัน &gt;</t>
   </si>
+  <si>
+    <t>Jones’ Salad 1 แถม 1  แค่ 3 วันเท่านั้น! 🧡 เฉพาะที่ ShopeeFood สั่งเลย! 👉🏻https://spf.shopee.co.th/AUr41VQfr6
+.
+✨ ต่อที่ 1: แรปทูน่าแซ่บ แถม แรปทูน่าคอร์น ลดเหลือ 159.-  จากปกติ 258.-
+✨ ต่อที่ 2: ใช้โค้ดลดเพิ่ม 23% สูงสุด 37.- (ขั้นต่ำ 150.-) เหลือ 123.-* (ตกชิ้นละ 62.-)  [เก็บโค้ดได้ที่หน้าร้าน]
+✨ ต่อที่ 3: ใช้ Coins ลดเพิ่มได้อีกสูงสุด 50% ของราคาอาหาร (สูงสุด 500 Coins ต่อวัน)
+. 
+📆 เฉพาะวันที่ 23 พ.ค. 69 - 25 พ.ค. 69 เท่านั้น
+*โค้ดส่วนลดมีจำนวนจำกัด อ่านเงื่อนไขเพิ่มเติมในหน้าร้านค้า, เฉพาะสาขาที่ร่วมรายการ</t>
+  </si>
+  <si>
+    <t>https://spf.shopee.co.th/AUr41VQfr6</t>
+  </si>
+  <si>
+    <t>23 พ.ค. 69 - 25 พ.ค. 69</t>
+  </si>
+  <si>
+    <t>https://scontent.fbkk5-3.fna.fbcdn.net/v/t45.1600-4/702603435_28929535299982147_3788639315739728465_n.jpg?stp=cp0_dst-jpg_q75_s640x640_sh2.08_spS444_tt6&amp;_nc_cat=111&amp;ccb=1-7&amp;_nc_sid=f0a831&amp;_nc_ohc=V2AwK-cNQ2cQ7kNvwHG_E27&amp;_nc_oc=Adq6zodVz10ySfSpgYzhAelbpm2FE9BfvkWP9--iVWP_DSq8hP_BV6GLZJXPsSvtOC78SMuQqrxx2es53BxEAXrD&amp;_nc_zt=1&amp;_nc_ht=scontent.fbkk5-3.fna&amp;_nc_gid=Flm83m6RInhXSiPa2r1J4g&amp;_nc_ss=7b2a8&amp;oh=00_Af6rB5coH6Rn6z85dAf32XP3Q8niuBtVEi-peo0cAltVZg&amp;oe=6A174B1F</t>
+  </si>
+  <si>
+    <t>https://s.shopee.co.th/7VDSS8caH8</t>
+  </si>
+  <si>
+    <t>💥 ทุบราคาลด 50% เที่ยงคืนและเที่ยงวัน
+25 พ.ค. 69 วันเดียวเท่านั้น รอช้อปเลย &gt;</t>
+  </si>
+  <si>
+    <t>https://scontent.fbkk5-7.fna.fbcdn.net/v/t45.1600-4/704660353_985573763852308_4918865503800114273_n.jpg?stp=cp0_dst-jpg_q75_s640x640_sh2.08_spS444_tt6&amp;_nc_cat=108&amp;ccb=1-7&amp;_nc_sid=f0a831&amp;_nc_ohc=1VzZr1rcXUkQ7kNvwGMsg80&amp;_nc_oc=AdoLm8A1vxktKREmcuqvDdJ5pvokG_3b46lXmLrcClRikg9rt_i_fu_jj_4oEi9VdbsYkIYk__c-p-5rox7ooDa3&amp;_nc_zt=1&amp;_nc_ht=scontent.fbkk5-7.fna&amp;_nc_gid=48DyjIlz9uWPAEnO9JGxew&amp;_nc_ss=7b2a8&amp;oh=00_Af70N8eGrKahNjdpJpccxGZmqtNfLDSTqQaAfOKLZlC2-A&amp;oe=6A172E7C</t>
+  </si>
+  <si>
+    <t>25 พ.ค. 69 วันเดียวเท่านั้น</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -363,6 +395,14 @@
     <font>
       <sz val="11"/>
       <name val="Arial"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="4">
@@ -422,7 +462,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -444,6 +484,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -930,8 +971,21 @@
       <c r="G5" t="s">
         <v>28</v>
       </c>
-      <c r="H5" s="8"/>
-      <c r="I5" s="3"/>
+      <c r="H5" s="8" t="s">
+        <v>97</v>
+      </c>
+      <c r="I5" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="J5" t="s">
+        <v>14</v>
+      </c>
+      <c r="K5" t="s">
+        <v>99</v>
+      </c>
+      <c r="L5" t="s">
+        <v>100</v>
+      </c>
     </row>
     <row r="6" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B6" s="6" t="s">
@@ -951,6 +1005,21 @@
       </c>
       <c r="G6" t="s">
         <v>32</v>
+      </c>
+      <c r="H6" s="8" t="s">
+        <v>102</v>
+      </c>
+      <c r="I6" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="J6" t="s">
+        <v>14</v>
+      </c>
+      <c r="K6" t="s">
+        <v>104</v>
+      </c>
+      <c r="L6" s="9" t="s">
+        <v>103</v>
       </c>
     </row>
     <row r="7" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -1262,8 +1331,11 @@
     <hyperlink ref="L3" display="https://scontent.fbkk5-5.fna.fbcdn.net/v/t39.30808-6/703381478_1431727098993056_7654736348316212425_n.jpg?_nc_cat=100&amp;ccb=1-7&amp;_nc_sid=127cfc&amp;_nc_ohc=UA_eHSY3CkoQ7kNvwEgdmDx&amp;_nc_oc=AdphnlCje5UXdWCWU-Q5bgZQPi_BeeX4EZrmC6ADIXQDlCQf0AR8p7CDqQiyEyORp5SF74M12uR"/>
     <hyperlink ref="I3" r:id="rId40"/>
     <hyperlink ref="I4" r:id="rId41"/>
-    <hyperlink ref="L4"/>
+    <hyperlink ref="L4" display="https://scontent.fbkk5-7.fna.fbcdn.net/v/t39.30808-6/704978599_1352491643674255_148307674156852835_n.jpg?_nc_cat=107&amp;ccb=1-7&amp;_nc_sid=127cfc&amp;_nc_ohc=TCbsBfpm4nsQ7kNvwGsGLDi&amp;_nc_oc=AdoX_rArGr5_WQu4JktN6gMRzm97hzElZXbhEDajLPJMb0ssLtBwTRke061UIq91ZFsm0ol7BJ_i"/>
+    <hyperlink ref="I5" r:id="rId42"/>
+    <hyperlink ref="I6" r:id="rId43"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId44"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add Dog Food, Auto Feeder, Litter Scoop, Dog Shirt, Dog Dryer, and Pet Wipes to affiliate products
</commit_message>
<xml_diff>
--- a/affiliate_products.xlsx
+++ b/affiliate_products.xlsx
@@ -507,7 +507,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L20"/>
+  <dimension ref="A1:L26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1323,6 +1323,186 @@
       <c r="F20" s="5" t="inlineStr">
         <is>
           <t>ลด 20% วันนี้เท่านั้น</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>4</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>พร้อมส่ง MJ.Kudson อาหารสุนัขพรีเมียมสูตรแกะ (ลดขนร่วง ลดคราบน้ำตา ลดกลิ่นมูลสัตว์) ทานได้ทุกสายพันธุ์</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/4ftKYsex7J</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>xxx</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>อาหารสุนัขเกรดพรีเมียมสูตรแกะ บำรุงขน ลดคราบน้ำตา</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>5</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>4-6L เครื่องให้อาหารสัตว์เลี้ยงอัตโนมัติ รองรับWiFi &amp; APP เครื่องให้อาหาร เครื่องให้อาหารแมวอัตโนมัติ สําหรับสัตว์เลี้ยง</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/LkLOw8JTI</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>xxx</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>เครื่องให้อาหารสัตว์เลี้ยงอัตโนมัติ 4-6L ควบคุมผ่านแอป WiFi</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>6</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>ตักทรายแมว ที่ตักอึแมว ตักขี้แมว ที่ตักทรายแมวสแตนเลส ตักง่ายล้างสะอาด เหมาะกับทรายทุกชนิด</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/1gFizQIzsN</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>xxx</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>ที่ตักทรายแมวสแตนเลส แข็งแรง ทนทาน ตักง่าย ทำความสะอาดสะดวก</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>7</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>เสื้อน้องหมาลาย เครื่องปรุงรส ผ้าไมโครสีสันสดใสพร้อมส่ง</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/1102CEXvU5</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>xxx</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>เสื้อน้องหมาลายเครื่องปรุงรสสุดกวน สีสันสดใส ผ้านุ่มสบาย</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>8</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>ไดร์เป่าขนสุนัข 2 มอเตอร์ ไดร์เป่าขนหมาใหญ่ เป่าผมสุนัข สัตว์เลี้ยง เครื่องเป่าขนสุนัข รุ่น A22-2300 | Haftigt</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/BQvCjV49w</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>xxx</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>ไดร์เป่าขนสุนัข 2 มอเตอร์ พลังลมแรง เป่าแห้งไวสำหรับสุนัขทุกขนาด</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>9</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>[พร้อมส่ง] EGG ทิชชู่เปียก Pet wipes 80 แผ่น ผ้าเช็ดตาและหูสัตว์เลี้ยง สำหรับเช็ดสัต ว์เลี้ยง ทิชชู่เปียก ทิชชู่หมา</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/3qKDZW3FKa</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>xxx</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>ทิชชู่เปียกสำหรับสัตว์เลี้ยง EGG Pet Wipes 80 แผ่น อ่อนโยน ปลอดภัย</t>
         </is>
       </c>
     </row>

</xml_diff>